<commit_message>
Auto update: 2026-03-07 07:02:19
</commit_message>
<xml_diff>
--- a/Listing/BAK02D.xlsx
+++ b/Listing/BAK02D.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="298">
   <si>
     <t/>
   </si>
@@ -295,6 +295,18 @@
     <t>SARI ROTI CKL-STRAWB</t>
   </si>
   <si>
+    <t>10018154</t>
+  </si>
+  <si>
+    <t>SARI ROTI TW.CHIP275</t>
+  </si>
+  <si>
+    <t>10004946</t>
+  </si>
+  <si>
+    <t>SARI ROTI COKL.VANLA</t>
+  </si>
+  <si>
     <t>20003593</t>
   </si>
   <si>
@@ -355,13 +367,34 @@
     <t>SR.ROTI SD CK.KJ 72</t>
   </si>
   <si>
+    <t>11</t>
+  </si>
+  <si>
     <t>20125603</t>
   </si>
   <si>
     <t>SR/RT SBK DUO COK 72</t>
   </si>
   <si>
-    <t>11</t>
+    <t>12</t>
+  </si>
+  <si>
+    <t>20137879</t>
+  </si>
+  <si>
+    <t>SARI KUE VAN.C 6'S</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>20137857</t>
+  </si>
+  <si>
+    <t>SARI KUE PND.C 6S</t>
+  </si>
+  <si>
+    <t>14</t>
   </si>
   <si>
     <t>20036000</t>
@@ -538,12 +571,6 @@
     <t>ARNON ROTI MESES 5'S</t>
   </si>
   <si>
-    <t>20129036</t>
-  </si>
-  <si>
-    <t>ARNON ROTI SSR CKLT</t>
-  </si>
-  <si>
     <t>20137768</t>
   </si>
   <si>
@@ -601,6 +628,12 @@
     <t>MR.BREAD CKLT KCNG</t>
   </si>
   <si>
+    <t>20069665</t>
+  </si>
+  <si>
+    <t>MR.BRD KSR CKLT KEJU</t>
+  </si>
+  <si>
     <t>20070168</t>
   </si>
   <si>
@@ -637,9 +670,6 @@
     <t>MR.BRD TAWAR TEBAL4S</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
     <t>20020008</t>
   </si>
   <si>
@@ -694,9 +724,6 @@
     <t>MR.BREAD TAWAR TEBAL</t>
   </si>
   <si>
-    <t>13</t>
-  </si>
-  <si>
     <t>20135734</t>
   </si>
   <si>
@@ -731,9 +758,6 @@
   </si>
   <si>
     <t>PRM BREAD COOKIES</t>
-  </si>
-  <si>
-    <t>14</t>
   </si>
   <si>
     <t>20100666</t>
@@ -1273,7 +1297,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2095,10 +2119,10 @@
         <v>3</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>5</v>
@@ -2118,7 +2142,7 @@
         <v>20</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>5</v>
@@ -2138,7 +2162,7 @@
         <v>20</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>5</v>
@@ -2158,7 +2182,7 @@
         <v>20</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>5</v>
@@ -2178,7 +2202,7 @@
         <v>20</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>5</v>
@@ -2198,7 +2222,7 @@
         <v>20</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>5</v>
@@ -2218,7 +2242,7 @@
         <v>20</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>5</v>
@@ -2238,7 +2262,7 @@
         <v>20</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>5</v>
@@ -2258,7 +2282,7 @@
         <v>20</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>5</v>
@@ -2278,7 +2302,7 @@
         <v>20</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>5</v>
@@ -2298,7 +2322,7 @@
         <v>20</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>5</v>
@@ -2306,19 +2330,19 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="C52" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>5</v>
@@ -2335,10 +2359,10 @@
         <v>3</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>4</v>
+        <v>121</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>5</v>
@@ -2346,19 +2370,19 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>5</v>
@@ -2366,19 +2390,19 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>8</v>
+        <v>127</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>5</v>
@@ -2386,10 +2410,10 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>3</v>
@@ -2398,7 +2422,7 @@
         <v>24</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>5</v>
@@ -2406,10 +2430,10 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>3</v>
@@ -2418,7 +2442,7 @@
         <v>24</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>5</v>
@@ -2426,10 +2450,10 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>3</v>
@@ -2438,7 +2462,7 @@
         <v>24</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>5</v>
@@ -2446,10 +2470,10 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>3</v>
@@ -2458,7 +2482,7 @@
         <v>24</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>5</v>
@@ -2466,10 +2490,10 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>3</v>
@@ -2478,7 +2502,7 @@
         <v>24</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>5</v>
@@ -2486,10 +2510,10 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>3</v>
@@ -2498,7 +2522,7 @@
         <v>24</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>5</v>
@@ -2506,10 +2530,10 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>3</v>
@@ -2518,7 +2542,7 @@
         <v>24</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>5</v>
@@ -2526,10 +2550,10 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>3</v>
@@ -2538,7 +2562,7 @@
         <v>24</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>5</v>
@@ -2546,10 +2570,10 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>3</v>
@@ -2558,7 +2582,7 @@
         <v>24</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>5</v>
@@ -2566,10 +2590,10 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>3</v>
@@ -2578,7 +2602,7 @@
         <v>24</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>5</v>
@@ -2586,10 +2610,10 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>3</v>
@@ -2598,7 +2622,7 @@
         <v>24</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>5</v>
@@ -2606,10 +2630,10 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>3</v>
@@ -2618,7 +2642,7 @@
         <v>24</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>5</v>
@@ -2626,10 +2650,10 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>3</v>
@@ -2638,7 +2662,7 @@
         <v>24</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F68" s="1" t="s">
         <v>5</v>
@@ -2646,10 +2670,10 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>3</v>
@@ -2658,7 +2682,7 @@
         <v>24</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F69" s="1" t="s">
         <v>5</v>
@@ -2666,10 +2690,10 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>3</v>
@@ -2678,7 +2702,7 @@
         <v>24</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>5</v>
@@ -2686,10 +2710,10 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>3</v>
@@ -2698,7 +2722,7 @@
         <v>24</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>5</v>
@@ -2706,10 +2730,10 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>3</v>
@@ -2718,7 +2742,7 @@
         <v>24</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>5</v>
@@ -2726,10 +2750,10 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>3</v>
@@ -2738,7 +2762,7 @@
         <v>24</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>5</v>
@@ -2746,19 +2770,19 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D74" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E74" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="E74" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>5</v>
@@ -2766,19 +2790,19 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D75" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E75" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>5</v>
@@ -2786,19 +2810,19 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="F76" s="1" t="s">
         <v>5</v>
@@ -2806,19 +2830,19 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>5</v>
@@ -2826,19 +2850,19 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>5</v>
@@ -2846,16 +2870,16 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>11</v>
@@ -2866,16 +2890,16 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>14</v>
@@ -2886,10 +2910,10 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>3</v>
@@ -2898,7 +2922,7 @@
         <v>48</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F81" s="1" t="s">
         <v>5</v>
@@ -2906,10 +2930,10 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>3</v>
@@ -2918,7 +2942,7 @@
         <v>48</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>5</v>
@@ -2926,19 +2950,19 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>5</v>
@@ -2946,19 +2970,19 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F84" s="1" t="s">
         <v>5</v>
@@ -2966,19 +2990,19 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>5</v>
@@ -2986,10 +3010,10 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>3</v>
@@ -2998,18 +3022,18 @@
         <v>51</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>187</v>
+        <v>5</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>3</v>
@@ -3018,7 +3042,7 @@
         <v>51</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>5</v>
@@ -3026,10 +3050,10 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>3</v>
@@ -3038,7 +3062,7 @@
         <v>51</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F88" s="1" t="s">
         <v>5</v>
@@ -3046,10 +3070,10 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>3</v>
@@ -3058,18 +3082,18 @@
         <v>51</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>5</v>
+        <v>196</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>3</v>
@@ -3078,7 +3102,7 @@
         <v>51</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F90" s="1" t="s">
         <v>5</v>
@@ -3086,19 +3110,19 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>5</v>
@@ -3106,39 +3130,39 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F93" s="1" t="s">
         <v>5</v>
@@ -3146,19 +3170,19 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>5</v>
@@ -3166,19 +3190,19 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F95" s="1" t="s">
         <v>5</v>
@@ -3186,39 +3210,39 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>208</v>
+        <v>118</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>208</v>
+        <v>118</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>5</v>
@@ -3226,19 +3250,19 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>208</v>
+        <v>118</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>5</v>
@@ -3246,19 +3270,19 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>208</v>
+        <v>118</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>5</v>
@@ -3266,19 +3290,19 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>208</v>
+        <v>121</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>5</v>
@@ -3286,19 +3310,19 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>208</v>
+        <v>121</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F101" s="1" t="s">
         <v>5</v>
@@ -3306,19 +3330,19 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>208</v>
+        <v>121</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>5</v>
@@ -3326,19 +3350,19 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>208</v>
+        <v>121</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="F103" s="1" t="s">
         <v>5</v>
@@ -3346,19 +3370,19 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>208</v>
+        <v>121</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>5</v>
@@ -3366,19 +3390,19 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>227</v>
+        <v>121</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>5</v>
@@ -3386,19 +3410,19 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>227</v>
+        <v>121</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>5</v>
@@ -3406,19 +3430,19 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>227</v>
+        <v>121</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>5</v>
@@ -3426,19 +3450,19 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>227</v>
+        <v>121</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>5</v>
@@ -3446,19 +3470,19 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>227</v>
+        <v>124</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>5</v>
@@ -3466,19 +3490,19 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>227</v>
+        <v>124</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F110" s="1" t="s">
         <v>5</v>
@@ -3486,19 +3510,19 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>240</v>
+        <v>124</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>5</v>
@@ -3515,10 +3539,10 @@
         <v>3</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>240</v>
+        <v>124</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F112" s="1" t="s">
         <v>5</v>
@@ -3535,10 +3559,10 @@
         <v>3</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>240</v>
+        <v>124</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>5</v>
@@ -3555,10 +3579,10 @@
         <v>3</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>240</v>
+        <v>124</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>5</v>
@@ -3575,10 +3599,10 @@
         <v>3</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>5</v>
@@ -3595,10 +3619,10 @@
         <v>3</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>5</v>
@@ -3615,10 +3639,10 @@
         <v>3</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>5</v>
@@ -3635,10 +3659,10 @@
         <v>3</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F118" s="1" t="s">
         <v>5</v>
@@ -3655,10 +3679,10 @@
         <v>3</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>116</v>
+        <v>17</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>5</v>
@@ -3675,10 +3699,10 @@
         <v>3</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>208</v>
+        <v>20</v>
       </c>
       <c r="F120" s="1" t="s">
         <v>5</v>
@@ -3695,10 +3719,10 @@
         <v>3</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>227</v>
+        <v>24</v>
       </c>
       <c r="F121" s="1" t="s">
         <v>5</v>
@@ -3715,10 +3739,10 @@
         <v>3</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>263</v>
+        <v>27</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>5</v>
@@ -3726,19 +3750,19 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B123" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="B123" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="C123" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E123" s="1" t="s">
-        <v>266</v>
+        <v>118</v>
       </c>
       <c r="F123" s="1" t="s">
         <v>5</v>
@@ -3746,19 +3770,19 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>269</v>
+        <v>121</v>
       </c>
       <c r="F124" s="1" t="s">
         <v>5</v>
@@ -3766,19 +3790,19 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>272</v>
+        <v>124</v>
       </c>
       <c r="F125" s="1" t="s">
         <v>5</v>
@@ -3786,19 +3810,19 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="F126" s="1" t="s">
         <v>5</v>
@@ -3806,19 +3830,19 @@
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>240</v>
+        <v>127</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="F127" s="1" t="s">
         <v>5</v>
@@ -3826,101 +3850,181 @@
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>281</v>
+        <v>127</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>4</v>
+        <v>277</v>
       </c>
       <c r="F128" s="1" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>281</v>
+        <v>127</v>
       </c>
       <c r="E129" s="1" t="s">
-        <v>8</v>
+        <v>280</v>
       </c>
       <c r="F129" s="1" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>281</v>
+        <v>127</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>11</v>
+        <v>283</v>
       </c>
       <c r="F130" s="1" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E131" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="B131" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C131" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D131" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="E131" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="F131" s="1" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="B132" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="B132" s="1" t="s">
+      <c r="C132" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D132" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="C132" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D132" s="1" t="s">
-        <v>281</v>
-      </c>
       <c r="E132" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D133" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="E133" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="E134" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="E135" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D136" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="E136" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F132" s="1" t="s">
+      <c r="F136" s="1" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>